<commit_message>
Add licence, reuse status, and access date to sources
</commit_message>
<xml_diff>
--- a/Dataset Sources.xlsx
+++ b/Dataset Sources.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F29C328-DE4B-41E9-8052-F3A557E1F301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5C1130-433F-4259-B6B9-91C6E0D7CEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19065" yWindow="5595" windowWidth="24540" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16665" yWindow="3945" windowWidth="24540" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Sources" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="76">
   <si>
     <t>Image Range</t>
   </si>
@@ -225,6 +225,27 @@
     <t>Unused images</t>
   </si>
   <si>
+    <t>License</t>
+  </si>
+  <si>
+    <t>CC BY 4.0</t>
+  </si>
+  <si>
+    <t>CC0 1.0 Universal</t>
+  </si>
+  <si>
+    <t>Used only for experimental model development; original images not redistributed</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Reuse Status</t>
+  </si>
+  <si>
+    <t>Allowed</t>
+  </si>
+  <si>
     <t>https://www.kaggle.com/datasets/abdullahkhanuet22/eggs-images-classification-damaged-or-not</t>
   </si>
   <si>
@@ -232,13 +253,16 @@
   </si>
   <si>
     <t>Classification</t>
+  </si>
+  <si>
+    <t>Access Date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -258,6 +282,11 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -306,7 +335,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -332,12 +361,54 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -452,8 +523,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DatasetSourcesTable" displayName="DatasetSourcesTable" ref="A1:M11" totalsRowShown="0">
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DatasetSourcesTable" displayName="DatasetSourcesTable" ref="A1:P11" totalsRowShown="0">
+  <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Image Range"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Dataset Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Owner"/>
@@ -461,12 +532,15 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Images Used"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Cracked Used"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Non-cracked Used"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Egg Colour" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Original Task" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Egg Colour" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Original Task" dataDxfId="4"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Re-annotated?"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Test/ Train" dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Unused images" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Test/ Train" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Unused images" dataDxfId="2"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Source URL"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="License" dataDxfId="1"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Reuse Status" dataDxfId="0" dataCellStyle="Hyperlink"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Access Date"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -667,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -683,9 +757,11 @@
     <col min="11" max="11" width="12.625" customWidth="1"/>
     <col min="12" max="12" width="8.375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="50" customWidth="1"/>
+    <col min="15" max="15" width="38.875" customWidth="1"/>
+    <col min="16" max="16" width="12.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -725,8 +801,17 @@
       <c r="M1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="N1" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="O1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="P1" t="s">
+        <v>75</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -766,8 +851,17 @@
       <c r="M2" s="4" t="s">
         <v>14</v>
       </c>
+      <c r="N2" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P2" s="11">
+        <v>45658</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -807,8 +901,17 @@
       <c r="M3" s="4" t="s">
         <v>18</v>
       </c>
+      <c r="N3" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="O3" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P3" s="11">
+        <v>45658</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -848,8 +951,17 @@
       <c r="M4" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="N4" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P4" s="11">
+        <v>45658</v>
+      </c>
     </row>
-    <row r="5" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
@@ -887,10 +999,19 @@
         <v>694</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P5" s="11">
+        <v>45689</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -916,7 +1037,7 @@
         <v>57</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>13</v>
@@ -930,8 +1051,17 @@
       <c r="M6" s="4" t="s">
         <v>30</v>
       </c>
+      <c r="N6" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="O6" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P6" s="11">
+        <v>45658</v>
+      </c>
     </row>
-    <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -971,8 +1101,17 @@
       <c r="M7" s="4" t="s">
         <v>34</v>
       </c>
+      <c r="N7" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="P7" s="11">
+        <v>45689</v>
+      </c>
     </row>
-    <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
@@ -1012,8 +1151,17 @@
       <c r="M8" s="4" t="s">
         <v>38</v>
       </c>
+      <c r="N8" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="O8" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P8" s="11">
+        <v>45658</v>
+      </c>
     </row>
-    <row r="9" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
@@ -1053,8 +1201,17 @@
       <c r="M9" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="N9" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="O9" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P9" s="11">
+        <v>45658</v>
+      </c>
     </row>
-    <row r="10" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
@@ -1080,7 +1237,7 @@
         <v>54</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>13</v>
@@ -1094,8 +1251,17 @@
       <c r="M10" s="4" t="s">
         <v>46</v>
       </c>
+      <c r="N10" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="O10" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="P10" s="11">
+        <v>45689</v>
+      </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>47</v>
       </c>
@@ -1120,6 +1286,8 @@
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
       <c r="M11" s="3"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Add per-source train/validation and test counts
</commit_message>
<xml_diff>
--- a/Dataset Sources.xlsx
+++ b/Dataset Sources.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5C1130-433F-4259-B6B9-91C6E0D7CEC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80CC5162-6B7B-4241-A320-68B270C9D937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16665" yWindow="3945" windowWidth="24540" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23040" yWindow="3090" windowWidth="24540" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Sources" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="74">
   <si>
     <t>Image Range</t>
   </si>
@@ -174,12 +174,6 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Test/ Train</t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
     <t>Original Task</t>
   </si>
   <si>
@@ -216,12 +210,6 @@
     <t>Egg object detection</t>
   </si>
   <si>
-    <t>Test and Train/ Val</t>
-  </si>
-  <si>
-    <t>Train/ Val</t>
-  </si>
-  <si>
     <t>Unused images</t>
   </si>
   <si>
@@ -246,16 +234,22 @@
     <t>Allowed</t>
   </si>
   <si>
+    <t>Used for Training/ Validation</t>
+  </si>
+  <si>
+    <t>Used for Testing</t>
+  </si>
+  <si>
+    <t>Egg detection</t>
+  </si>
+  <si>
+    <t>Classification</t>
+  </si>
+  <si>
+    <t>Access Date</t>
+  </si>
+  <si>
     <t>https://www.kaggle.com/datasets/abdullahkhanuet22/eggs-images-classification-damaged-or-not</t>
-  </si>
-  <si>
-    <t>Egg detection</t>
-  </si>
-  <si>
-    <t>Classification</t>
-  </si>
-  <si>
-    <t>Access Date</t>
   </si>
 </sst>
 </file>
@@ -335,7 +329,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -358,9 +352,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -368,12 +359,68 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <fill>
@@ -484,31 +531,6 @@
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -523,8 +545,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DatasetSourcesTable" displayName="DatasetSourcesTable" ref="A1:P11" totalsRowShown="0">
-  <tableColumns count="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DatasetSourcesTable" displayName="DatasetSourcesTable" ref="A1:Q11" totalsRowShown="0">
+  <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Image Range"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Dataset Name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Owner"/>
@@ -532,14 +554,15 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Images Used"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Cracked Used"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Non-cracked Used"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Egg Colour" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Original Task" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Egg Colour" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Original Task" dataDxfId="5"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Re-annotated?"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Test/ Train" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Unused images" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Used for Training/ Validation" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Used for Testing" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Unused images" dataDxfId="0"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Source URL"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="License" dataDxfId="1"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Reuse Status" dataDxfId="0" dataCellStyle="Hyperlink"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="License" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Reuse Status" dataDxfId="2" dataCellStyle="Hyperlink"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Access Date"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -741,7 +764,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -754,14 +777,16 @@
     <col min="8" max="8" width="12.125" customWidth="1"/>
     <col min="9" max="9" width="14.375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.625" customWidth="1"/>
-    <col min="12" max="12" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="50" customWidth="1"/>
-    <col min="15" max="15" width="38.875" customWidth="1"/>
-    <col min="16" max="16" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.75" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="50" customWidth="1"/>
+    <col min="15" max="15" width="9.5" customWidth="1"/>
+    <col min="16" max="16" width="38.875" customWidth="1"/>
+    <col min="17" max="17" width="12.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -784,34 +809,37 @@
         <v>6</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="M1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="O1" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="P1" t="s">
-        <v>75</v>
+        <v>61</v>
+      </c>
+      <c r="P1" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -834,34 +862,37 @@
         <v>0</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="6">
+        <v>50</v>
+      </c>
+      <c r="L2" s="6">
+        <v>20</v>
+      </c>
+      <c r="M2" s="11">
+        <v>7</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="L2" s="8">
-        <v>7</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="N2" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="O2" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="P2" s="11">
+      <c r="P2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q2" s="10">
         <v>45658</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -884,34 +915,37 @@
         <v>160</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="6">
+        <v>580</v>
+      </c>
+      <c r="L3" s="6">
+        <v>65</v>
+      </c>
+      <c r="M3" s="11">
+        <v>3836</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O3" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="L3" s="8">
-        <v>3836</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N3" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="O3" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="P3" s="11">
+      <c r="P3" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q3" s="10">
         <v>45658</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -934,34 +968,37 @@
         <v>100</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="6">
+        <v>80</v>
+      </c>
+      <c r="L4" s="6">
+        <v>20</v>
+      </c>
+      <c r="M4" s="11">
+        <v>41</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="L4" s="8">
-        <v>41</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="O4" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="P4" s="11">
+      <c r="P4" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q4" s="10">
         <v>45658</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>23</v>
       </c>
@@ -984,34 +1021,37 @@
         <v>85</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="L5" s="8">
+      <c r="K5" s="6">
+        <v>0</v>
+      </c>
+      <c r="L5" s="6">
+        <v>100</v>
+      </c>
+      <c r="M5" s="11">
         <v>694</v>
       </c>
-      <c r="M5" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="N5" s="9" t="s">
+      <c r="N5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="P5" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="O5" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="P5" s="11">
+      <c r="Q5" s="10">
         <v>45689</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>27</v>
       </c>
@@ -1034,34 +1074,37 @@
         <v>55</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K6" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="L6" s="8">
+      <c r="K6" s="6">
+        <v>55</v>
+      </c>
+      <c r="L6" s="6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="11">
         <v>735</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="N6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="N6" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="O6" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="P6" s="11">
+      <c r="O6" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="P6" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q6" s="10">
         <v>45658</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -1084,34 +1127,37 @@
         <v>0</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="L7" s="8">
+      <c r="K7" s="6">
+        <v>80</v>
+      </c>
+      <c r="L7" s="6">
+        <v>0</v>
+      </c>
+      <c r="M7" s="11">
         <v>11218</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="N7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="N7" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="O7" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="P7" s="11">
+      <c r="O7" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q7" s="10">
         <v>45689</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
@@ -1134,34 +1180,37 @@
         <v>0</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="L8" s="8">
+      <c r="K8" s="6">
+        <v>0</v>
+      </c>
+      <c r="L8" s="6">
+        <v>50</v>
+      </c>
+      <c r="M8" s="11">
         <v>2020</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="N8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="N8" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="O8" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="P8" s="11">
+      <c r="O8" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="P8" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q8" s="10">
         <v>45658</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
@@ -1184,34 +1233,37 @@
         <v>40</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="6">
+        <v>35</v>
+      </c>
+      <c r="L9" s="6">
+        <v>5</v>
+      </c>
+      <c r="M9" s="11">
+        <v>1394</v>
+      </c>
+      <c r="N9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="O9" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="L9" s="8">
-        <v>1394</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="N9" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="O9" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="P9" s="11">
+      <c r="P9" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q9" s="10">
         <v>45658</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
@@ -1234,34 +1286,37 @@
         <v>260</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="K10" s="6">
+        <v>240</v>
+      </c>
+      <c r="L10" s="6">
+        <v>20</v>
+      </c>
+      <c r="M10" s="11">
+        <v>1789</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="O10" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="L10" s="8">
-        <v>1789</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="N10" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="O10" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="P10" s="11">
+      <c r="P10" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q10" s="10">
         <v>45689</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>47</v>
       </c>
@@ -1283,23 +1338,30 @@
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="3"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="7"/>
+      <c r="K11" s="7">
+        <f>SUM(K2:K10)</f>
+        <v>1120</v>
+      </c>
+      <c r="L11" s="7">
+        <f>SUM(L2:L10)</f>
+        <v>280</v>
+      </c>
+      <c r="M11" s="12"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="M2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="M3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="M4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="M5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="M6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="M7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="M8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="M9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="M10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="N2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId10"/>

</xml_diff>